<commit_message>
reran h-chains and iron
</commit_message>
<xml_diff>
--- a/hydrogen_comps/rerun/H12_chain/H12_2.49/H12_2.49_energies.xlsx
+++ b/hydrogen_comps/rerun/H12_chain/H12_2.49/H12_2.49_energies.xlsx
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.0054789562</v>
+        <v>-0.0054793184</v>
       </c>
     </row>
     <row r="3">
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-6.00597003</v>
+        <v>-6.00597004</v>
       </c>
     </row>
     <row r="4">
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-6.01144899</v>
+        <v>-6.01144936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>